<commit_message>
Update AI systems report materials
</commit_message>
<xml_diff>
--- a/outputs/ai_complex_systems_materials/数据与模型附录.xlsx
+++ b/outputs/ai_complex_systems_materials/数据与模型附录.xlsx
@@ -7,10 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="行业应用指数" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="情景预测" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资料来源" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型说明" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Industry_Maturity" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario_Forecast" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk_Matrix" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -174,7 +176,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>行业AI综合应用指数</a:t>
+              <a:t>Industry AI Maturity Index</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -189,7 +191,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'行业应用指数'!G1</f>
+              <f>'Industry_Maturity'!H1</f>
             </strRef>
           </tx>
           <spPr>
@@ -199,12 +201,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'行业应用指数'!$A$2:$A$7</f>
+              <f>'Industry_Maturity'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'行业应用指数'!$G$2:$G$7</f>
+              <f>'Industry_Maturity'!$H$2:$H$9</f>
             </numRef>
           </val>
         </ser>
@@ -218,21 +220,6 @@
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>指数</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -254,7 +241,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>行业</a:t>
+                  <a:t>AMI</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -286,7 +273,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>2030年前AI驱动产出指数情景</a:t>
+              <a:t>AI Output Scenario</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -298,9 +285,6 @@
         <ser>
           <idx val="0"/>
           <order val="0"/>
-          <tx>
-            <v>保守情景</v>
-          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -316,21 +300,18 @@
           </marker>
           <cat>
             <numRef>
-              <f>'情景预测'!$B$2:$B$4</f>
+              <f>'Scenario_Forecast'!$B$2:$B$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'情景预测'!$C$2:$C$4</f>
+              <f>'Scenario_Forecast'!$C$2:$C$7</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="1"/>
           <order val="1"/>
-          <tx>
-            <v>基准情景</v>
-          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -346,21 +327,18 @@
           </marker>
           <cat>
             <numRef>
-              <f>'情景预测'!$B$2:$B$4</f>
+              <f>'Scenario_Forecast'!$B$2:$B$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'情景预测'!$C$5:$C$7</f>
+              <f>'Scenario_Forecast'!$C$8:$C$13</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="2"/>
           <order val="2"/>
-          <tx>
-            <v>积极情景</v>
-          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -376,12 +354,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'情景预测'!$B$2:$B$4</f>
+              <f>'Scenario_Forecast'!$B$2:$B$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'情景预测'!$C$8:$C$10</f>
+              <f>'Scenario_Forecast'!$C$14:$C$19</f>
             </numRef>
           </val>
         </ser>
@@ -403,7 +381,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>年份</a:t>
+                  <a:t>Year</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -430,7 +408,122 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>产出指数</a:t>
+                  <a:t>Index</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Risk Matrix</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <scatterChart>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>Risk</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'Risk_Matrix'!$B$2:$B$7</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Risk_Matrix'!$C$2:$C$7</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Probability</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="20"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Impact</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -454,7 +547,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>9</col>
+      <col>12</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
@@ -481,12 +574,39 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>8</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5400000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4680000" cy="2880000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -793,17 +913,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -829,20 +952,35 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>流程重构</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>利润改善潜力</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>社会影响权重</t>
-        </is>
-      </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>综合应用指数</t>
+          <t>社会价值</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>AMI</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>合规摩擦</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>价值潜力</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>典型场景</t>
         </is>
@@ -851,90 +989,117 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>先进制造</t>
+          <t>金融科技</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>0.68</v>
+        <v>0.83</v>
       </c>
       <c r="C2" s="2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="F2" s="2" t="n">
         <v>0.78</v>
       </c>
-      <c r="D2" s="2" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="E2" s="2" t="n">
+      <c r="G2" s="2" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="I2" s="2" t="n">
         <v>0.62</v>
       </c>
-      <c r="F2" s="2" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>质检、预测性维护、排产优化、数字孪生</t>
+      <c r="J2" s="2" t="n">
+        <v>0.585</v>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>风控、反欺诈、智能投研、运营自动化</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>金融科技</t>
+          <t>先进制造</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0.82</v>
+        <v>0.72</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.74</v>
+        <v>0.79</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.76</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>0.71</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.61</v>
+        <v>0.74</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>风控、智能投顾、反欺诈、运营自动化</t>
+        <v>0.58</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0.724</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>0.549</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>质量检测、预测性维护、柔性排产、数字孪生</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>气象环境</t>
+          <t>能源电力</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>0.57</v>
+        <v>0.66</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.74</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.64</v>
+        <v>0.73</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.53</v>
+        <v>0.67</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>0.7</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>短临预报、灾害预警、污染扩散模拟</t>
+        <v>0.72</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>0.702</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>0.517</v>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>负荷预测、电网调度、设备巡检、能效优化</t>
         </is>
       </c>
     </row>
@@ -945,86 +1110,191 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>0.61</v>
+        <v>0.64</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.72</v>
+        <v>0.78</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.66</v>
+        <v>0.68</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.55</v>
+        <v>0.59</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.46</v>
+        <v>0.62</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>医学影像、临床文书、药物发现</t>
+        <v>0.76</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>0.675</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>0.452</v>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>医学影像、临床文书、药物发现、分诊辅助</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>交通物流</t>
+          <t>气象环境</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0.59</v>
+        <v>0.6</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.63</v>
+        <v>0.7</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0.58</v>
+        <v>0.62</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.52</v>
+        <v>0.55</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>路径优化、仓储调度、自动驾驶辅助</t>
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>0.657</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>短临预报、灾害预警、污染扩散模拟</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>交通物流</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>0.469</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>路径优化、仓储调度、交通流预测、辅助驾驶</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
           <t>教育与知识服务</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D7" s="2" t="n">
+      <c r="B8" s="2" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="D8" s="2" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="E7" s="2" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>个性化学习、内容生成、知识检索</t>
+      <c r="E8" s="2" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>0.624</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>0.388</v>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>个性化学习、知识检索、内容生成、学习评估</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>政务与公共服务</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>0.609</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>0.378</v>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>智能问答、审批辅助、城市治理、公共安全预警</t>
         </is>
       </c>
     </row>
@@ -1040,15 +1310,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1064,29 +1335,34 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>综合产出指数(2025=100)</t>
+          <t>综合产出指数</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>AI年生产率贡献百分点</t>
+          <t>年生产率贡献百分点</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>AI采用率假设</t>
+          <t>AI采用率</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>人机协同任务占比</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>AI资本形成占比</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>保守情景</t>
+          <t>审慎扩散</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -1096,129 +1372,147 @@
         <v>100</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.4</v>
+        <v>0.42</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0.45</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.53</v>
+        <v>0.52</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0.24</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>保守情景</t>
+          <t>审慎扩散</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>108.3</v>
+        <v>105</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.4</v>
+        <v>0.42</v>
       </c>
       <c r="E3" s="2" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="F3" s="2" t="n">
         <v>0.55</v>
       </c>
-      <c r="F3" s="2" t="n">
-        <v>0.57</v>
+      <c r="G3" s="2" t="n">
+        <v>0.25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>保守情景</t>
+          <t>审慎扩散</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>2030</v>
+        <v>2027</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>121.7</v>
+        <v>110.1</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.4</v>
+        <v>0.42</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.65</v>
+        <v>0.6</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.61</v>
+        <v>0.58</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>0.27</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>基准情景</t>
+          <t>审慎扩散</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2025</v>
+        <v>2028</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>100</v>
+        <v>115.4</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.8</v>
+        <v>0.42</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.45</v>
+        <v>0.66</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.53</v>
+        <v>0.6</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>0.29</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>基准情景</t>
+          <t>审慎扩散</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>2027</v>
+        <v>2029</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>112.5</v>
+        <v>121</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.8</v>
+        <v>0.42</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0.7</v>
+        <v>0.71</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.64</v>
+        <v>0.62</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>基准情景</t>
+          <t>审慎扩散</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
         <v>2030</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>135.2</v>
+        <v>126.9</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.8</v>
+        <v>0.42</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0.85</v>
+        <v>0.76</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.71</v>
+        <v>0.64</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0.32</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>积极情景</t>
+          <t>基准转化</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -1228,57 +1522,291 @@
         <v>100</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1.3</v>
+        <v>0.82</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>0.45</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.53</v>
+        <v>0.52</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0.24</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>积极情景</t>
+          <t>基准转化</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>118.9</v>
+        <v>107.4</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>1.3</v>
+        <v>0.82</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0.76</v>
+        <v>0.58</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.58</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0.28</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>积极情景</t>
+          <t>基准转化</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
+        <v>2027</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>116.2</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>基准转化</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>2028</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>126.2</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>基准转化</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>2029</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>137.4</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>基准转化</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
         <v>2030</v>
       </c>
-      <c r="C10" s="2" t="n">
-        <v>154.4</v>
-      </c>
-      <c r="D10" s="2" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="E10" s="2" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="F10" s="2" t="n">
-        <v>0.79</v>
+      <c r="C13" s="2" t="n">
+        <v>149.5</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>加速协同</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>加速协同</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>110.2</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>加速协同</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>2027</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>123.3</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>加速协同</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>2028</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>139.1</v>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>0.46</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>加速协同</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>2029</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>157</v>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>0.52</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>加速协同</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>2030</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>177.6</v>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>0.57</v>
       </c>
     </row>
   </sheetData>
@@ -1293,203 +1821,359 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="72" customWidth="1" min="4" max="4"/>
-    <col width="58" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>编号</t>
+          <t>项目</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>机构</t>
+          <t>行业</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>资料</t>
+          <t>预算需求</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>关键摘录</t>
+          <t>算力需求</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>链接</t>
+          <t>人才需求</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>经济净现值</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>社会价值</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>风险系数</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>战略匹配</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>价值/成本</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>制造视觉质检与预测维护</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Stanford HAI</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>2025 AI Index Report</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>2024年美国私人AI投资1091亿美元；中国93亿美元；英国45亿美元。全球生成式AI私人投资339亿美元，同比+18.7%；组织AI使用率由2023年55%升至2024年78%。</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://hai.stanford.edu/ai-index/2025-ai-index-report</t>
-        </is>
+          <t>先进制造</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>3.82</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>金融风控图谱与智能审查</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>McKinsey</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>The state of AI in 2025</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>2025年88%的受访组织在至少一个业务职能中常规使用AI；62%至少开始试验AI Agent；仅39%报告企业层面EBIT影响。</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mckinsey.com/capabilities/quantumblack/our-insights/the-state-of-ai</t>
-        </is>
+          <t>金融科技</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>3.6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>电网负荷预测与巡检智能体</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>World Economic Forum</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Future of Jobs Report 2025</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>到2030年宏观趋势预计创造1.70亿个岗位、替代9200万个岗位，净增7800万个；AI与信息处理技术预计创造1100万个并替代900万个岗位。</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.weforum.org/publications/the-future-of-jobs-report-2025/</t>
-        </is>
+          <t>能源电力</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>3.83</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>医疗影像与临床文书助手</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>OECD.AI</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Macroeconomic productivity gains from AI in G7 economies</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>在高AI暴露且采用更充分的经济体中，AI对年劳动生产率增速的贡献情景约为0.4-1.3个百分点。</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>https://oecd.ai/en/ai-publications/macroeconomic-productivity-gains-from-artificial-intelligence-in-g7-economies</t>
-        </is>
+          <t>医疗健康</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>3.04</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>S5</t>
+          <t>气象灾害短临预报系统</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>国务院</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>关于深入实施“人工智能+”行动的意见</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>到2027年新一代智能终端、智能体等应用普及率超过70%；到2030年超过90%，智能经济成为重要增长极。</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.gov.cn/zhengce/content/202508/content_7037861.htm</t>
-        </is>
+          <t>气象环境</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>3.77</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>S6</t>
+          <t>物流路径与仓储调度优化</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>工信部公开信息/中国新闻网转引</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>2025年中国人工智能核心产业规模预计突破1.2万亿元</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>2025年中国AI企业数量超过6000家，核心产业规模预计突破1.2万亿元人民币。</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>https://news.china.com.cn/2026-01/22/content_118293631.shtml</t>
-        </is>
+          <t>交通物流</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>3.97</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>知识服务检索增强平台</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>教育与知识服务</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>3.75</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>政务服务智能问答与审批辅助</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>政务与公共服务</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>3.47</v>
       </c>
     </row>
   </sheetData>
@@ -1503,82 +2187,467 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="100" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>模块</t>
+          <t>参数</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>说明</t>
+          <t>低位扰动</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>高位扰动</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>应用成熟度指数</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>0.25×渗透率 + 0.20×投资强度 + 0.20×数据可得性 + 0.20×利润改善潜力 + 0.15×社会影响权重</t>
-        </is>
+          <t>采用率上限</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>-8.6</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>10.9</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>随机森林</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>以AI投入、数据质量、流程重构、人才结构等为特征，识别生产率和利润率变化的关键因素。</t>
-        </is>
+          <t>数据质量</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>-7.3</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>MCMC</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>围绕采用率、生产率贡献和人机协同任务占比设定先验分布，模拟未来路径不确定性。</t>
-        </is>
+          <t>流程重构效率</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>9.1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>LP / CP-SAT</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>在预算、算力、人才和风险约束下，最大化AI项目组合的经济与社会价值。</t>
-        </is>
+          <t>算力成本</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>-5.8</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>4.2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>注意</t>
+          <t>合规摩擦</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>-4.9</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>5.3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>人才供给</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>-4.1</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="64" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>风险</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>概率</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>影响</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>治理建议</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>模型幻觉与错误决策</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>高风险场景必须保留人工复核与可追溯日志</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>数据偏差与分配不公</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>建立数据漂移监测、样本审计和公平性指标</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>隐私泄露与合规责任</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>采用最小化采集、脱敏、权限分层和审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>投资过热与收益不达预期</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>分阶段投资，以里程碑触发扩容</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>岗位任务重组摩擦</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>将再培训预算纳入项目可行性评价</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>供应商锁定与技术债</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>优先开放接口、可迁移模型和多云容灾</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
+    <col width="58" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>编号</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>机构</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>资料</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>关键摘录</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>链接</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Stanford HAI</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>AI Index Report 2025</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>组织AI使用率由2023年的55%升至2024年的78%；美国私人AI投资约1091亿美元。</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://hai.stanford.edu/ai-index/2025-ai-index-report</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>McKinsey</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>The State of AI in 2025</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>88%的受访组织在至少一个业务职能中常规使用AI，企业级收益仍依赖组织重构。</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mckinsey.com/capabilities/quantumblack/our-insights/the-state-of-ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>World Economic Forum</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Future of Jobs Report 2025</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>预计到2030年宏观趋势创造1.70亿个岗位、替代9200万个岗位，净增7800万个岗位。</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.weforum.org/publications/the-future-of-jobs-report-2025/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>OECD.AI</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Macroeconomic productivity gains from AI in G7 economies</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>不同采用速度下，AI对劳动生产率增速的额外贡献可形成多情景区间。</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://oecd.ai/en/ai-publications/macroeconomic-productivity-gains-from-artificial-intelligence-in-g7-economies</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>S5</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>本表为课程测算和展示用附录，不应表述为官方原始统计数据。</t>
+          <t>国务院</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>关于深入实施“人工智能+”行动的意见</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>提出推动人工智能与经济社会各行业各领域广泛深度融合，强调智能体和行业应用普及。</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gov.cn/zhengce/content/202508/content_7037861.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>工信部公开信息</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>人工智能产业公开资料</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>中国人工智能企业和核心产业规模快速扩张，形成应用供给侧基础。</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.miit.gov.cn/</t>
         </is>
       </c>
     </row>

</xml_diff>